<commit_message>
feat: add BTMA textile standards, update BSIA CS
</commit_message>
<xml_diff>
--- a/data/xlsx/bsia--smart-systems-engineering-embedded-design-and-semiconductor-application-interfaces.xlsx
+++ b/data/xlsx/bsia--smart-systems-engineering-embedded-design-and-semiconductor-application-interfaces.xlsx
@@ -99,7 +99,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="bottom"/>
@@ -132,6 +132,30 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -497,7 +521,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G38"/>
+  <dimension ref="A1:G41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15.17" customWidth="1" min="1" max="1"/>
@@ -569,7 +593,7 @@
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>Embedded/electronics lab (approx. for 25 trainees) with benches, storage and stationery</t>
+          <t>Computer Lab (400 sft) and Electronics Workshop/Laboratory (700–800 sft) for 25 trainees</t>
         </is>
       </c>
       <c r="D8" s="11" t="n"/>
@@ -634,12 +658,12 @@
       </c>
     </row>
     <row r="16" ht="14.15" customHeight="1">
-      <c r="A16" s="7" t="n">
+      <c r="A16" s="20" t="n">
         <v>1</v>
       </c>
       <c r="B16" s="8" t="inlineStr">
         <is>
-          <t>Computer/Laptop (1 unit) — trainer station</t>
+          <t>Computer/Laptop (Trainer)</t>
         </is>
       </c>
       <c r="C16" s="9" t="n">
@@ -658,12 +682,12 @@
       <c r="G16" s="9" t="n"/>
     </row>
     <row r="17" ht="14.15" customHeight="1">
-      <c r="A17" s="7" t="n">
+      <c r="A17" s="20" t="n">
         <v>2</v>
       </c>
       <c r="B17" s="8" t="inlineStr">
         <is>
-          <t>Multimedia projector &amp; screen (1 unit)</t>
+          <t>Printer</t>
         </is>
       </c>
       <c r="C17" s="9" t="n">
@@ -673,7 +697,7 @@
         <v>0</v>
       </c>
       <c r="E17" s="9" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="F17" s="9">
         <f>IFERROR(MIN(C17,D17)*E17/C17,0)</f>
@@ -682,12 +706,12 @@
       <c r="G17" s="9" t="n"/>
     </row>
     <row r="18" ht="14.15" customHeight="1">
-      <c r="A18" s="7" t="n">
+      <c r="A18" s="20" t="n">
         <v>3</v>
       </c>
       <c r="B18" s="8" t="inlineStr">
         <is>
-          <t>Printer (1 unit)</t>
+          <t>Multimedia Projector</t>
         </is>
       </c>
       <c r="C18" s="9" t="n">
@@ -697,7 +721,7 @@
         <v>0</v>
       </c>
       <c r="E18" s="9" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="F18" s="9">
         <f>IFERROR(MIN(C18,D18)*E18/C18,0)</f>
@@ -706,12 +730,12 @@
       <c r="G18" s="9" t="n"/>
     </row>
     <row r="19" ht="14.15" customHeight="1">
-      <c r="A19" s="7" t="n">
+      <c r="A19" s="20" t="n">
         <v>4</v>
       </c>
       <c r="B19" s="8" t="inlineStr">
         <is>
-          <t>Desktop/Laptop workstations (25 units) with internet access</t>
+          <t>High-performance Desktop/Laptop</t>
         </is>
       </c>
       <c r="C19" s="9" t="n">
@@ -730,22 +754,22 @@
       <c r="G19" s="9" t="n"/>
     </row>
     <row r="20" ht="14.15" customHeight="1">
-      <c r="A20" s="7" t="n">
+      <c r="A20" s="20" t="n">
         <v>5</v>
       </c>
       <c r="B20" s="8" t="inlineStr">
         <is>
-          <t>Embedded / electronics laboratory (for 25 trainees)</t>
+          <t>Embedded IDE and Toolchain Software (Arduino IDE / STM32CubeIDE / PlatformIO or equivalent)</t>
         </is>
       </c>
       <c r="C20" s="9" t="n">
-        <v>1</v>
+        <v>25</v>
       </c>
       <c r="D20" s="9" t="n">
         <v>0</v>
       </c>
       <c r="E20" s="9" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="F20" s="9">
         <f>IFERROR(MIN(C20,D20)*E20/C20,0)</f>
@@ -754,22 +778,22 @@
       <c r="G20" s="9" t="n"/>
     </row>
     <row r="21" ht="14.15" customHeight="1">
-      <c r="A21" s="7" t="n">
+      <c r="A21" s="20" t="n">
         <v>6</v>
       </c>
       <c r="B21" s="8" t="inlineStr">
         <is>
-          <t>Embedded development boards — Arduino, ESP32, STM32, Raspberry Pi Pico or equivalent (per trainee)</t>
+          <t>EDA/PCB Design Software (Schematic Capture and PCB Layout)</t>
         </is>
       </c>
       <c r="C21" s="9" t="n">
-        <v>1</v>
+        <v>25</v>
       </c>
       <c r="D21" s="9" t="n">
         <v>0</v>
       </c>
       <c r="E21" s="9" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F21" s="9">
         <f>IFERROR(MIN(C21,D21)*E21/C21,0)</f>
@@ -778,12 +802,12 @@
       <c r="G21" s="9" t="n"/>
     </row>
     <row r="22" ht="14.15" customHeight="1">
-      <c r="A22" s="7" t="n">
+      <c r="A22" s="20" t="n">
         <v>7</v>
       </c>
       <c r="B22" s="8" t="inlineStr">
         <is>
-          <t>Embedded IDEs / toolchains — Arduino IDE, PlatformIO, STM32CubeIDE, Wokwi or vendor SDK (25)</t>
+          <t>MCU Development Boards (STM32 / ESP32 / Arduino / RP2040 or equivalent)</t>
         </is>
       </c>
       <c r="C22" s="9" t="n">
@@ -802,16 +826,16 @@
       <c r="G22" s="9" t="n"/>
     </row>
     <row r="23" ht="14.15" customHeight="1">
-      <c r="A23" s="7" t="n">
+      <c r="A23" s="20" t="n">
         <v>8</v>
       </c>
       <c r="B23" s="8" t="inlineStr">
         <is>
-          <t>Sensor modules — temperature, humidity, motion/IMU, current, light/optical, environmental</t>
+          <t>Sensor and Interface Module Kits (Temperature, Humidity, Pressure, IMU, Light, Gas, Display, Relay, etc.)</t>
         </is>
       </c>
       <c r="C23" s="9" t="n">
-        <v>1</v>
+        <v>25</v>
       </c>
       <c r="D23" s="9" t="n">
         <v>0</v>
@@ -826,22 +850,22 @@
       <c r="G23" s="9" t="n"/>
     </row>
     <row r="24" ht="14.15" customHeight="1">
-      <c r="A24" s="7" t="n">
+      <c r="A24" s="20" t="n">
         <v>9</v>
       </c>
       <c r="B24" s="8" t="inlineStr">
         <is>
-          <t>Communication/interface modules and displays (OLED/LCD; UART/I2C/SPI/RS232/RS485)</t>
+          <t>Breadboard and Electronic Component Kits</t>
         </is>
       </c>
       <c r="C24" s="9" t="n">
-        <v>1</v>
+        <v>25</v>
       </c>
       <c r="D24" s="9" t="n">
         <v>0</v>
       </c>
       <c r="E24" s="9" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="F24" s="9">
         <f>IFERROR(MIN(C24,D24)*E24/C24,0)</f>
@@ -850,12 +874,12 @@
       <c r="G24" s="9" t="n"/>
     </row>
     <row r="25" ht="14.15" customHeight="1">
-      <c r="A25" s="7" t="n">
+      <c r="A25" s="20" t="n">
         <v>10</v>
       </c>
       <c r="B25" s="8" t="inlineStr">
         <is>
-          <t>PCB design tools — KiCad, EasyEDA, Altium or equivalent EDA tools (25)</t>
+          <t>JTAG/SWD Debugger/Programmer</t>
         </is>
       </c>
       <c r="C25" s="9" t="n">
@@ -874,22 +898,22 @@
       <c r="G25" s="9" t="n"/>
     </row>
     <row r="26" ht="14.15" customHeight="1">
-      <c r="A26" s="7" t="n">
+      <c r="A26" s="20" t="n">
         <v>11</v>
       </c>
       <c r="B26" s="8" t="inlineStr">
         <is>
-          <t>Digital oscilloscope (per bench)</t>
+          <t>Digital Multimeter</t>
         </is>
       </c>
       <c r="C26" s="9" t="n">
-        <v>1</v>
+        <v>25</v>
       </c>
       <c r="D26" s="9" t="n">
         <v>0</v>
       </c>
       <c r="E26" s="9" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F26" s="9">
         <f>IFERROR(MIN(C26,D26)*E26/C26,0)</f>
@@ -898,22 +922,22 @@
       <c r="G26" s="9" t="n"/>
     </row>
     <row r="27" ht="14.15" customHeight="1">
-      <c r="A27" s="7" t="n">
+      <c r="A27" s="20" t="n">
         <v>12</v>
       </c>
       <c r="B27" s="8" t="inlineStr">
         <is>
-          <t>Logic analyzer with protocol decoding (per bench)</t>
+          <t>ESD-safe Workbench with ESD Mat and Wrist Strap</t>
         </is>
       </c>
       <c r="C27" s="9" t="n">
-        <v>1</v>
+        <v>25</v>
       </c>
       <c r="D27" s="9" t="n">
         <v>0</v>
       </c>
       <c r="E27" s="9" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="F27" s="9">
         <f>IFERROR(MIN(C27,D27)*E27/C27,0)</f>
@@ -922,16 +946,16 @@
       <c r="G27" s="9" t="n"/>
     </row>
     <row r="28" ht="14.15" customHeight="1">
-      <c r="A28" s="7" t="n">
+      <c r="A28" s="20" t="n">
         <v>13</v>
       </c>
       <c r="B28" s="8" t="inlineStr">
         <is>
-          <t>JTAG/SWD debugger (per bench)</t>
+          <t>Digital Storage Oscilloscope</t>
         </is>
       </c>
       <c r="C28" s="9" t="n">
-        <v>1</v>
+        <v>13</v>
       </c>
       <c r="D28" s="9" t="n">
         <v>0</v>
@@ -946,22 +970,22 @@
       <c r="G28" s="9" t="n"/>
     </row>
     <row r="29" ht="14.15" customHeight="1">
-      <c r="A29" s="7" t="n">
+      <c r="A29" s="20" t="n">
         <v>14</v>
       </c>
       <c r="B29" s="8" t="inlineStr">
         <is>
-          <t>Digital multimeters and adjustable power supplies (per bench)</t>
+          <t>Logic Analyzer</t>
         </is>
       </c>
       <c r="C29" s="9" t="n">
-        <v>1</v>
+        <v>13</v>
       </c>
       <c r="D29" s="9" t="n">
         <v>0</v>
       </c>
       <c r="E29" s="9" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F29" s="9">
         <f>IFERROR(MIN(C29,D29)*E29/C29,0)</f>
@@ -970,22 +994,22 @@
       <c r="G29" s="9" t="n"/>
     </row>
     <row r="30" ht="14.15" customHeight="1">
-      <c r="A30" s="7" t="n">
+      <c r="A30" s="20" t="n">
         <v>15</v>
       </c>
       <c r="B30" s="8" t="inlineStr">
         <is>
-          <t>Semiconductor devices — MCUs, sensor ICs, LDO/switching regulators, MOSFETs, level shifters, ESD protection</t>
+          <t>DC Regulated Power Supply</t>
         </is>
       </c>
       <c r="C30" s="9" t="n">
-        <v>1</v>
+        <v>13</v>
       </c>
       <c r="D30" s="9" t="n">
         <v>0</v>
       </c>
       <c r="E30" s="9" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="F30" s="9">
         <f>IFERROR(MIN(C30,D30)*E30/C30,0)</f>
@@ -994,22 +1018,22 @@
       <c r="G30" s="9" t="n"/>
     </row>
     <row r="31" ht="14.15" customHeight="1">
-      <c r="A31" s="7" t="n">
+      <c r="A31" s="20" t="n">
         <v>16</v>
       </c>
       <c r="B31" s="8" t="inlineStr">
         <is>
-          <t>Breadboards, prototyping boards, basic components and hand tools</t>
+          <t>Soldering Station with Fume Extractor</t>
         </is>
       </c>
       <c r="C31" s="9" t="n">
-        <v>1</v>
+        <v>13</v>
       </c>
       <c r="D31" s="9" t="n">
         <v>0</v>
       </c>
       <c r="E31" s="9" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F31" s="9">
         <f>IFERROR(MIN(C31,D31)*E31/C31,0)</f>
@@ -1018,22 +1042,22 @@
       <c r="G31" s="9" t="n"/>
     </row>
     <row r="32" ht="14.15" customHeight="1">
-      <c r="A32" s="7" t="n">
+      <c r="A32" s="20" t="n">
         <v>17</v>
       </c>
       <c r="B32" s="8" t="inlineStr">
         <is>
-          <t>Soldering and assembly stations with ESD protection (per bench)</t>
+          <t>Function Generator</t>
         </is>
       </c>
       <c r="C32" s="9" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D32" s="9" t="n">
         <v>0</v>
       </c>
       <c r="E32" s="9" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F32" s="9">
         <f>IFERROR(MIN(C32,D32)*E32/C32,0)</f>
@@ -1042,16 +1066,16 @@
       <c r="G32" s="9" t="n"/>
     </row>
     <row r="33" ht="14.15" customHeight="1">
-      <c r="A33" s="7" t="n">
+      <c r="A33" s="20" t="n">
         <v>18</v>
       </c>
       <c r="B33" s="8" t="inlineStr">
         <is>
-          <t>PPE, ESD mat and wrist strap; first-aid and fire-safety equipment</t>
+          <t>Current Probe/Power Profiling Tool</t>
         </is>
       </c>
       <c r="C33" s="9" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D33" s="9" t="n">
         <v>0</v>
@@ -1066,12 +1090,12 @@
       <c r="G33" s="9" t="n"/>
     </row>
     <row r="34" ht="14.15" customHeight="1">
-      <c r="A34" s="7" t="n">
+      <c r="A34" s="20" t="n">
         <v>19</v>
       </c>
       <c r="B34" s="8" t="inlineStr">
         <is>
-          <t>Serial terminals, USB-serial adapters and cabling</t>
+          <t>PCB Prototype Fabrication and Assembly Support (In-house or Outsourced)</t>
         </is>
       </c>
       <c r="C34" s="9" t="n">
@@ -1081,65 +1105,145 @@
         <v>0</v>
       </c>
       <c r="E34" s="9" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F34" s="9">
         <f>IFERROR(MIN(C34,D34)*E34/C34,0)</f>
         <v/>
       </c>
-      <c r="G34" s="9" t="n"/>
-    </row>
-    <row r="35">
-      <c r="A35" s="10" t="inlineStr">
+      <c r="G34" s="9" t="inlineStr">
+        <is>
+          <t>01 set</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="14.15" customHeight="1">
+      <c r="A35" s="20" t="n">
+        <v>20</v>
+      </c>
+      <c r="B35" s="8" t="inlineStr">
+        <is>
+          <t>Internet Connectivity with Network Switch and Router</t>
+        </is>
+      </c>
+      <c r="C35" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="D35" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E35" s="9" t="n">
+        <v>5</v>
+      </c>
+      <c r="F35" s="9">
+        <f>IFERROR(MIN(C35,D35)*E35/C35,0)</f>
+        <v/>
+      </c>
+      <c r="G35" s="9" t="n"/>
+    </row>
+    <row r="36" ht="14.15" customHeight="1">
+      <c r="A36" s="20" t="n">
+        <v>21</v>
+      </c>
+      <c r="B36" s="8" t="inlineStr">
+        <is>
+          <t>Central File/Storage Server</t>
+        </is>
+      </c>
+      <c r="C36" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="D36" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E36" s="9" t="n">
+        <v>5</v>
+      </c>
+      <c r="F36" s="9">
+        <f>IFERROR(MIN(C36,D36)*E36/C36,0)</f>
+        <v/>
+      </c>
+      <c r="G36" s="9" t="n"/>
+    </row>
+    <row r="37" ht="14.15" customHeight="1">
+      <c r="A37" s="20" t="n">
+        <v>22</v>
+      </c>
+      <c r="B37" s="8" t="inlineStr">
+        <is>
+          <t>First Aid and Fire Safety Equipment</t>
+        </is>
+      </c>
+      <c r="C37" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="D37" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E37" s="9" t="n">
+        <v>5</v>
+      </c>
+      <c r="F37" s="9">
+        <f>IFERROR(MIN(C37,D37)*E37/C37,0)</f>
+        <v/>
+      </c>
+      <c r="G37" s="9" t="inlineStr">
+        <is>
+          <t>01 set</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="21" t="inlineStr">
         <is>
           <t>Sum</t>
-        </is>
-      </c>
-      <c r="B35" s="11" t="n"/>
-      <c r="C35" s="11" t="n"/>
-      <c r="D35" s="12" t="n"/>
-      <c r="E35" s="10">
-        <f>SUM(E16:E34)</f>
-        <v/>
-      </c>
-      <c r="F35" s="10">
-        <f>SUM(F16:F34)</f>
-        <v/>
-      </c>
-      <c r="G35" s="13" t="n"/>
-    </row>
-    <row r="36">
-      <c r="A36" s="10" t="inlineStr">
-        <is>
-          <t>Score out of 100</t>
-        </is>
-      </c>
-      <c r="B36" s="11" t="n"/>
-      <c r="C36" s="11" t="n"/>
-      <c r="D36" s="11" t="n"/>
-      <c r="E36" s="12" t="n"/>
-      <c r="F36" s="10">
-        <f>F35/E35*100</f>
-        <v/>
-      </c>
-      <c r="G36" s="13" t="n"/>
-    </row>
-    <row r="37" ht="9.75" customHeight="1"/>
-    <row r="38">
-      <c r="A38" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Total achieved points out of 30  </t>
         </is>
       </c>
       <c r="B38" s="11" t="n"/>
       <c r="C38" s="11" t="n"/>
-      <c r="D38" s="11" t="n"/>
-      <c r="E38" s="12" t="n"/>
-      <c r="F38" s="10">
-        <f>F36*30/100</f>
-        <v/>
-      </c>
-      <c r="G38" s="10" t="inlineStr">
+      <c r="D38" s="12" t="n"/>
+      <c r="E38" s="21">
+        <f>SUM(E16:E37)</f>
+        <v/>
+      </c>
+      <c r="F38" s="21">
+        <f>SUM(F16:F37)</f>
+        <v/>
+      </c>
+      <c r="G38" s="13" t="n"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="21" t="inlineStr">
+        <is>
+          <t>Score out of 100</t>
+        </is>
+      </c>
+      <c r="B39" s="11" t="n"/>
+      <c r="C39" s="11" t="n"/>
+      <c r="D39" s="11" t="n"/>
+      <c r="E39" s="12" t="n"/>
+      <c r="F39" s="21">
+        <f>F38/E38*100</f>
+        <v/>
+      </c>
+      <c r="G39" s="13" t="n"/>
+    </row>
+    <row r="40" ht="9.75" customHeight="1"/>
+    <row r="41">
+      <c r="A41" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Total achieved points out of 30  </t>
+        </is>
+      </c>
+      <c r="B41" s="11" t="n"/>
+      <c r="C41" s="11" t="n"/>
+      <c r="D41" s="11" t="n"/>
+      <c r="E41" s="12" t="n"/>
+      <c r="F41" s="21">
+        <f>F39*30/100</f>
+        <v/>
+      </c>
+      <c r="G41" s="21" t="inlineStr">
         <is>
           <t>Points</t>
         </is>
@@ -1148,13 +1252,13 @@
   </sheetData>
   <mergeCells count="8">
     <mergeCell ref="A13:G13"/>
+    <mergeCell ref="A39:E39"/>
     <mergeCell ref="C7:G7"/>
     <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A38:E38"/>
-    <mergeCell ref="A35:D35"/>
-    <mergeCell ref="A36:E36"/>
+    <mergeCell ref="A40:G40"/>
+    <mergeCell ref="A38:D38"/>
+    <mergeCell ref="A41:E41"/>
     <mergeCell ref="C8:G8"/>
-    <mergeCell ref="A37:G37"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>